<commit_message>
Plantillas de carga masiva alineadas a las 3 categorías del motor de precios
Los selectores de plantilla ahora dicen Ropa/Tecnología/Joyería (antes
Joyería/Cosmético/Lencería) para que coincidan exactamente con las
categorías que tienen margen propio en /admin/precios. Cada plantilla
trae su ejemplo con la columna Categoría ya llena con ese nombre, así
que descargar y subir sin editarla calcula el precio con el % correcto
desde el primer intento. Se retira Cosmético del selector (sin
categoría de margen equivalente) y su lógica de columnas específicas
(volumen/fragancia) en el validador.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/plantillas/joyeria.xlsx
+++ b/public/plantillas/joyeria.xlsx
@@ -502,7 +502,7 @@
         <v>Anillo solitario diamante</v>
       </c>
       <c r="H2" t="str">
-        <v>Anillos</v>
+        <v>Joyería</v>
       </c>
       <c r="I2" t="str">
         <v>local</v>
@@ -561,7 +561,7 @@
         <v>Cadena básica 45cm</v>
       </c>
       <c r="H3" t="str">
-        <v>Cadenas</v>
+        <v>Joyería</v>
       </c>
       <c r="I3" t="str">
         <v>local</v>

</xml_diff>